<commit_message>
docs: update sprint plan for completed reporting work
</commit_message>
<xml_diff>
--- a/docs/08_sprint_plan.xlsx
+++ b/docs/08_sprint_plan.xlsx
@@ -3862,10 +3862,14 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>reporting-refresh</t>
+        </is>
+      </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
           <t>Should</t>
@@ -3881,7 +3885,11 @@
           <t>Reporting &amp; Analytics</t>
         </is>
       </c>
-      <c r="G49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>PMT bands chart and horizontal household distribution now live.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3891,10 +3899,14 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>reporting-refresh</t>
+        </is>
+      </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
           <t>Should</t>
@@ -3910,7 +3922,11 @@
           <t>Reporting &amp; Analytics</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Pipeline funnel and DRS status views now live.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3920,10 +3936,14 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>reporting-refresh</t>
+        </is>
+      </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
           <t>Must</t>
@@ -3939,7 +3959,11 @@
           <t>Reporting &amp; Analytics</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Dedup status views and DQA violation record downloads now live.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3949,10 +3973,14 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>reporting-refresh</t>
+        </is>
+      </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
           <t>Should</t>
@@ -3968,7 +3996,11 @@
           <t>Reporting &amp; Analytics</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Weekly registrations/submissions trends, export controls, and role-aware error states now live.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -6064,7 +6096,6 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr">
         <is>
           <t>Must</t>
@@ -6097,7 +6128,6 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr"/>
       <c r="D117" t="inlineStr">
         <is>
           <t>Must</t>
@@ -6130,7 +6160,6 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr">
         <is>
           <t>Must</t>
@@ -6163,7 +6192,6 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr">
         <is>
           <t>Must</t>
@@ -6196,7 +6224,6 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr">
         <is>
           <t>Should</t>
@@ -7401,7 +7428,7 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>45 of 114 stories</t>
+          <t>49 of 114 stories</t>
         </is>
       </c>
     </row>
@@ -7423,10 +7450,8 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>62</t>
-        </is>
+      <c r="B21" s="10" t="n">
+        <v>58</v>
       </c>
     </row>
     <row r="22">
@@ -7469,7 +7494,7 @@
       <c r="A27" s="9" t="inlineStr"/>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>12 backlog stories are partial — they have scaffolds but UI wiring or polish is pending.</t>
+          <t>7 backlog stories are partial — they have scaffolds but UI wiring or polish is pending, and the reporting surface now includes live dashboards, exports, and record-level drill-downs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(docs): record S27 (UPD history tabs + SRM role) in sprint plan
Status sheet + Story Map rows for today's session. The file is broadly
stale (S4 still marked "in progress" while we're at S26+ per dpia/);
this just captures what landed today, not a backfill.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/08_sprint_plan.xlsx
+++ b/docs/08_sprint_plan.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story Map" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog Status" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forward" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Status" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Story Map" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Backlog Status" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Forward" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Dependencies" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Notes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Story Map'!$A$1:$F$45</definedName>
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +57,10 @@
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="9">
@@ -128,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -159,6 +163,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -525,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -808,6 +818,36 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>S27</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>26 May EAT</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>~1 hour</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>UPD workbench history view: Decided + On-hold tabs on the change-request screen, manual ?status= filter on /api/v1/upd/change-requests/ (django-filter no-op workaround), Social Registry Manager role added to Tweaks role switcher for approver-persona demos. 5 new pytest filter tests; full UPD suite + 204 JS tests green.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -819,7 +859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2267,6 +2307,70 @@
       <c r="F45" s="2" t="inlineStr">
         <is>
           <t>pip-audit + bandit configuration + ruff cleanup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>S27/srm-role</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>(pending)</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>(design persona)</t>
+        </is>
+      </c>
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>SEC, UPD</t>
+        </is>
+      </c>
+      <c r="F46" s="11" t="inlineStr">
+        <is>
+          <t>Social Registry Manager added to Tweaks role switcher — approver persona for demoing AC-UPD-NO-SELF-APPROVE flows without swapping accounts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>S27/upd-history-tabs</t>
+        </is>
+      </c>
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>(pending)</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D47" s="11" t="inlineStr">
+        <is>
+          <t>US-S22-001</t>
+        </is>
+      </c>
+      <c r="E47" s="11" t="inlineStr">
+        <is>
+          <t>UPD</t>
+        </is>
+      </c>
+      <c r="F47" s="11" t="inlineStr">
+        <is>
+          <t>Decided + On-hold tabs on the change-request workbench. Manual ?status= filter in ChangeRequestViewSet.get_queryset() — filterset_fields was silently a no-op (django-filter not installed). +5 pytest filter tests.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(docs): backfill sprint plan with S5..S26 + post-S26 iterations
The XLSX had been stale since S4 in-progress (15 May). Backfill from
dpia/sprint_*.md (S5..S26) plus git log for S20/S21 (which have no
dpia file — minimal personal-data surface). S26b row consolidates
the post-2026-05-21 work landed today across six commits: PMT
rejection-terminal, PMT Configuration live wiring, unified Approvals
queue, admin-screen polish, user manual scaffold, source-of-truth
audit. Story Map gets a sprint-level pointer row per sprint (granular
US-story tracking already lives in dpia/sprint_*.md).

S4 was also flipped to Done — that work (partner ABAC, NUSAF
connector, routing matrix → REF-DATA) shipped long ago and the
"in progress" marker had decayed.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/08_sprint_plan.xlsx
+++ b/docs/08_sprint_plan.xlsx
@@ -132,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -169,6 +169,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -535,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -706,12 +709,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>15 May 09:53 → … EAT</t>
+          <t>15 May 2026</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -724,7 +727,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Partner-side ABAC on API-DRS, NUSAF connector, routing matrix → REF-DATA (UPD-O-01 resolved).</t>
+          <t>Partner-side ABAC on API-DRS, NUSAF connector, routing matrix → REF-DATA (UPD-O-01 resolved). Subsumed into S5+ sprint sequence.</t>
         </is>
       </c>
     </row>
@@ -845,6 +848,678 @@
       <c r="F10" s="11" t="inlineStr">
         <is>
           <t>UPD workbench history view: Decided + On-hold tabs on the change-request screen, manual ?status= filter on /api/v1/upd/change-requests/ (django-filter no-op workaround), Social Registry Manager role added to Tweaks role switcher for approver-persona demos. 5 new pytest filter tests; full UPD suite + 204 JS tests green.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>S5+S6</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>~1 day</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>~30</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>UPD ChangeRequest admin workbench (US-S5-001), API-DRS export-bundle render (US-S5-002), DDUP merge REVERSED state (US-S5-003), DIH WFP SCOPE connector (US-S5-004), IDV NIRA queue+retry (US-S5-005), API-DRS expiry sweep (US-S5-006). See dpia/sprint_5_6_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>~half day</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>~15</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>UPD auto-escalation on SLA breach, DIH NIRA reverse-feed (vital events), DDUP tier 3 probabilistic discovery, DRS partner /requests/mine/, RPT CSV exports, ADR-0006 Keycloak realm. See dpia/sprint_7_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>~half day</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>~12</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>DDUP tier-3 auto-merge confidence rule, DRS partner download endpoint, RPT weekly registrations dashboard, DIH connector framework, GRM workbench (first React screen). See dpia/sprint_8_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>~half day</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>~12</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>DDUP MatchPair admin per_field_scores, RPT grievances-by-category dashboard, DRS throttling, GRM → UPD cross-screen handoff, DRS partner portal screen. See dpia/sprint_9_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>S10+S11</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>~1 day</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>~20</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>Tweaks panel reopen pill, DDUP reverse-merge counters, Partner DRS request-builder (third React screen), UPD bulk-action endpoints, DIH ConnectorRun admin. See dpia/sprint_10_11_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>~half day</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>~10</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Home-screen KPIs from live counts, live Audit chain + Updates history tabs on household detail, Celery beat for pending Kobo landings. See dpia/sprint_12_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>~half day</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>~10</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Adopt claude.ai Registry + Household redesign, wire home queue panels live, DDUP screen live, DRS partner list live. See dpia/sprint_13_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>~half day</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>~10</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Merge-via-REST + DDUP React Merge loop, DRS operator list live, Programmes + Grievances tabs on household detail, per-region home drill-down. See dpia/sprint_14_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>~half day</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>~8</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>DDUP merge modal "Reversible until &lt;date&gt;", DRS operator avg decision turnaround, region drill-down extended to queue panels, ADR-0008 pagination+throttling sweep. See dpia/sprint_15_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>~half day</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>~8</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>Audit-reason enrichment, partner DRS typical wait time, Member endpoint max_page_size cap, audit-chain integrity scheduled job. See dpia/sprint_16_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>S17+S18</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>~1 day</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>~15</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>DDUP merge modal per-field similarity, home dashboard drill-down breadcrumb, DRS partner builder DSA-driven field disabling, US-082b RPT violations dashboard, US-082c failures_7d on DqaRule. See dpia/sprint_17_18_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>~1 day</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>~15</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>ChoiceList + ChoiceOption catalogue (US-116), FormSection/Question/SkipLogic/Constraint models (US-117a), questionnaire builder admin UI (US-117b), XLSForm export (US-118), rule-pack sync (US-119), legacy questionnaire import (US-120). See dpia/sprint_19_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>~half day</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>~6</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>PII-shape lint for constraint messages (US-S20-001), gate SQLite-only audit-chain tests on Postgres CI (US-S20-003), push FormVersion xlsx to Kobo (US-S20-004), lock active forms + clone-to-new-draft (US-S20-005), wire XLSForm geo selects to GeographicUnit (US-S20-006). (No dpia file — minimal personal-data surface.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>~half day</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>~6</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>GRM workbench live API wiring (US-S21-002), GrievanceTask + resolve gate (US-S21-003), task visibility scoping (US-S21-004), persist + display resolve/close narrative (US-S21-005), Kobo missing-calculation fix (US-S21-006). (No dpia file — minimal personal-data surface.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>S22</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>~1 day</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>~25</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>UPD workbench live + Open-CR modal (US-S22-001..004), drop TextChoices on coded fields + resolver/serializer label fields + bundle endpoint + JSX wiring (US-S22-005a..g), connectors + registry JSX + UPD field-catalog corrections (US-S22-005h..j). See dpia/sprint_22_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>S22-DE</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>~1 day</t>
+        </is>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>~15</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>Detail entities — 14 new tables capturing per-section questionnaire repeats (health, education, employment, dwelling, utilities, food, shock, coping). Special-category data review per DPPA 2019 §§9–10. See dpia/sprint_22_detail_entities_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>~1 day</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>~15</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>Partners module — Partner + PartnerContact models (US-S23-004..005), DataSharingAgreement + DsaSignature (US-S23-006), signature workflow (US-S23-010), PartnerUsageDaily + activity projection (US-S23-007), API surface (US-S23-008..009), lint gate + e2e tests (US-S23-014..015). See dpia/sprint_23_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>S24</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>~half day</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>~6</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>Canonical Partner + DSA consolidation — lift DRS-local rows to apps.partners (US-S24-002), schema swap + canonical enforcement (US-S24-003..004). See dpia/sprint_24_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>~half day</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>~5</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>Programme registration wizard — ChoiceLists seeded (US-S25-001), Programme model extension (US-S25-002), CRUD endpoint (US-S25-003), wizard JSX wired to live API (US-S25-004), lint gate + integration tests (US-S25-005). See dpia/sprint_25_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>S26</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>~half day</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>~8</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>apps.referral.Programme consolidation — ADR-0015 (US-S26-001), referral_status ChoiceList seeded (US-S26-002), strip TextChoices + align enrolment codes (US-S26-003), lift Programme rows to canonical (US-S26-004), schema swap + drop legacy (US-S26-005), /api/v1/beneficiaries/ listing (US-S26-006). See dpia/sprint_26_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>S26b</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>2026-05-21 → 2026-05-26</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>~5 days</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>~80</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>Post-S26 iterations consolidated in this backfill: chatbot module (US-CHB-001..006), Open-CR modal slices (member picker, supporting docs, step wizard, before/after diff), DIH walk-in path + Quality-Failed archive + inline correction + reprocess workflow, source-of-truth audit, user manual mkdocs scaffold, refdata duplicate cleanup, home dashboard wiring fixes, chatbot Assistant in admin console, PMT signoff rejection terminal + PMT Configuration live wiring + unified Approvals queue. (Several commits not US-tagged — see git log.)</t>
         </is>
       </c>
     </row>
@@ -859,7 +1534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2371,6 +3046,934 @@
       <c r="F47" s="11" t="inlineStr">
         <is>
           <t>Decided + On-hold tabs on the change-request workbench. Manual ?status= filter in ChangeRequestViewSet.get_queryset() — filterset_fields was silently a no-op (django-filter not installed). +5 pytest filter tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>S5+S6/all</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C48" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>US-S5-001..006</t>
+        </is>
+      </c>
+      <c r="E48" s="11" t="inlineStr">
+        <is>
+          <t>UPD, API-DRS, DDUP, DIH, IDV</t>
+        </is>
+      </c>
+      <c r="F48" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_5_6_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
+        <is>
+          <t>S7/all</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C49" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr">
+        <is>
+          <t>US-S7-001..006</t>
+        </is>
+      </c>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>UPD, DIH, DDUP, DRS, RPT, SEC</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_7_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>S8/all</t>
+        </is>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C50" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>US-S8-001..006</t>
+        </is>
+      </c>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>DDUP, DRS, RPT, DIH, GRM</t>
+        </is>
+      </c>
+      <c r="F50" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_8_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>S9/all</t>
+        </is>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C51" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="inlineStr">
+        <is>
+          <t>US-S9-001..006</t>
+        </is>
+      </c>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t>DDUP, RPT, DRS, GRM, UPD</t>
+        </is>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_9_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t>S10+S11/all</t>
+        </is>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C52" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t>US-S10-001..006</t>
+        </is>
+      </c>
+      <c r="E52" s="11" t="inlineStr">
+        <is>
+          <t>design, DDUP, DRS, UPD, DIH</t>
+        </is>
+      </c>
+      <c r="F52" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_10_11_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="11" t="inlineStr">
+        <is>
+          <t>S12/all</t>
+        </is>
+      </c>
+      <c r="B53" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C53" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D53" s="11" t="inlineStr">
+        <is>
+          <t>US-S12-001..005</t>
+        </is>
+      </c>
+      <c r="E53" s="11" t="inlineStr">
+        <is>
+          <t>design, household, DIH</t>
+        </is>
+      </c>
+      <c r="F53" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_12_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>S13/all</t>
+        </is>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>US-S13-001..005</t>
+        </is>
+      </c>
+      <c r="E54" s="11" t="inlineStr">
+        <is>
+          <t>design, home, DDUP, DRS</t>
+        </is>
+      </c>
+      <c r="F54" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_13_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="inlineStr">
+        <is>
+          <t>S14/all</t>
+        </is>
+      </c>
+      <c r="B55" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr">
+        <is>
+          <t>US-S14-001..005</t>
+        </is>
+      </c>
+      <c r="E55" s="11" t="inlineStr">
+        <is>
+          <t>DDUP, DRS, household, home</t>
+        </is>
+      </c>
+      <c r="F55" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_14_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t>S15/all</t>
+        </is>
+      </c>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C56" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>US-S15-001..005</t>
+        </is>
+      </c>
+      <c r="E56" s="11" t="inlineStr">
+        <is>
+          <t>DDUP, DRS, home, API</t>
+        </is>
+      </c>
+      <c r="F56" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_15_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>S16/all</t>
+        </is>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="inlineStr">
+        <is>
+          <t>US-S16-001..005</t>
+        </is>
+      </c>
+      <c r="E57" s="11" t="inlineStr">
+        <is>
+          <t>SEC, DRS, DAT, audit</t>
+        </is>
+      </c>
+      <c r="F57" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_16_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>S17+S18/all</t>
+        </is>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C58" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>US-082b/c, US-S18-001..003</t>
+        </is>
+      </c>
+      <c r="E58" s="11" t="inlineStr">
+        <is>
+          <t>DAT-DQA, design, DDUP, DRS</t>
+        </is>
+      </c>
+      <c r="F58" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_17_18_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>S19/all</t>
+        </is>
+      </c>
+      <c r="B59" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C59" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D59" s="11" t="inlineStr">
+        <is>
+          <t>US-116..120</t>
+        </is>
+      </c>
+      <c r="E59" s="11" t="inlineStr">
+        <is>
+          <t>REF-DATA, INT, DAT-DQA</t>
+        </is>
+      </c>
+      <c r="F59" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_19_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>S20/all</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>(git)</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>US-S20-001/003..006</t>
+        </is>
+      </c>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>INT, SEC, REF-DATA</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>XLSForm + Kobo push + audit-test CI gate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>S21/all</t>
+        </is>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>(git)</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D61" s="11" t="inlineStr">
+        <is>
+          <t>US-S21-002..006</t>
+        </is>
+      </c>
+      <c r="E61" s="11" t="inlineStr">
+        <is>
+          <t>GRM, INT</t>
+        </is>
+      </c>
+      <c r="F61" s="11" t="inlineStr">
+        <is>
+          <t>GRM workbench live + GrievanceTask + resolve gate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>S22/all</t>
+        </is>
+      </c>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>US-S22-001..005</t>
+        </is>
+      </c>
+      <c r="E62" s="11" t="inlineStr">
+        <is>
+          <t>UPD, REF-DATA, design</t>
+        </is>
+      </c>
+      <c r="F62" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_22_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t>S22-DE/all</t>
+        </is>
+      </c>
+      <c r="B63" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C63" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D63" s="11" t="inlineStr">
+        <is>
+          <t>US-S22-DE</t>
+        </is>
+      </c>
+      <c r="E63" s="11" t="inlineStr">
+        <is>
+          <t>DAT (detail entities)</t>
+        </is>
+      </c>
+      <c r="F63" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_22_detail_entities_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>S23/all</t>
+        </is>
+      </c>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C64" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>US-S23-004..015</t>
+        </is>
+      </c>
+      <c r="E64" s="11" t="inlineStr">
+        <is>
+          <t>partners, SEC</t>
+        </is>
+      </c>
+      <c r="F64" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_23_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="11" t="inlineStr">
+        <is>
+          <t>S24/all</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C65" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D65" s="11" t="inlineStr">
+        <is>
+          <t>US-S24-002..004</t>
+        </is>
+      </c>
+      <c r="E65" s="11" t="inlineStr">
+        <is>
+          <t>partners</t>
+        </is>
+      </c>
+      <c r="F65" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_24_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>S25/all</t>
+        </is>
+      </c>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C66" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D66" s="11" t="inlineStr">
+        <is>
+          <t>US-S25-001..005</t>
+        </is>
+      </c>
+      <c r="E66" s="11" t="inlineStr">
+        <is>
+          <t>referral, design</t>
+        </is>
+      </c>
+      <c r="F66" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_25_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="11" t="inlineStr">
+        <is>
+          <t>S26/all</t>
+        </is>
+      </c>
+      <c r="B67" s="11" t="inlineStr">
+        <is>
+          <t>(dpia)</t>
+        </is>
+      </c>
+      <c r="C67" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D67" s="11" t="inlineStr">
+        <is>
+          <t>US-S26-001..006</t>
+        </is>
+      </c>
+      <c r="E67" s="11" t="inlineStr">
+        <is>
+          <t>referral, REF-DATA, beneficiaries</t>
+        </is>
+      </c>
+      <c r="F67" s="11" t="inlineStr">
+        <is>
+          <t>See dpia/sprint_26_impacts.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>S26b/chatbot</t>
+        </is>
+      </c>
+      <c r="B68" s="11" t="inlineStr">
+        <is>
+          <t>(this backfill)</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D68" s="11" t="inlineStr">
+        <is>
+          <t>US-CHB-001..006</t>
+        </is>
+      </c>
+      <c r="E68" s="11" t="inlineStr">
+        <is>
+          <t>chatbot</t>
+        </is>
+      </c>
+      <c r="F68" s="11" t="inlineStr">
+        <is>
+          <t>RAG over user manuals; Anthropic + sentence-transformers; ADR-0021.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="11" t="inlineStr">
+        <is>
+          <t>S26b/open-cr-modal</t>
+        </is>
+      </c>
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>(this backfill)</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D69" s="11" t="inlineStr">
+        <is>
+          <t>(UPD UI slices)</t>
+        </is>
+      </c>
+      <c r="E69" s="11" t="inlineStr">
+        <is>
+          <t>UPD, design</t>
+        </is>
+      </c>
+      <c r="F69" s="11" t="inlineStr">
+        <is>
+          <t>Member picker, supporting docs, step wizard, before/after diff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>S26b/dih-walkin</t>
+        </is>
+      </c>
+      <c r="B70" s="11" t="inlineStr">
+        <is>
+          <t>(this backfill)</t>
+        </is>
+      </c>
+      <c r="C70" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D70" s="11" t="inlineStr">
+        <is>
+          <t>(DIH UX iterations)</t>
+        </is>
+      </c>
+      <c r="E70" s="11" t="inlineStr">
+        <is>
+          <t>DIH</t>
+        </is>
+      </c>
+      <c r="F70" s="11" t="inlineStr">
+        <is>
+          <t>Walk-in submit + Quality-Failed archive + inline correction + reprocess workflow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="11" t="inlineStr">
+        <is>
+          <t>S26b/user-manual</t>
+        </is>
+      </c>
+      <c r="B71" s="11" t="inlineStr">
+        <is>
+          <t>(this backfill)</t>
+        </is>
+      </c>
+      <c r="C71" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D71" s="11" t="inlineStr">
+        <is>
+          <t>(docs)</t>
+        </is>
+      </c>
+      <c r="E71" s="11" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F71" s="11" t="inlineStr">
+        <is>
+          <t>mkdocs-material scaffold under /docs/user-manual served via Django /manual/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="11" t="inlineStr">
+        <is>
+          <t>S26b/source-of-truth</t>
+        </is>
+      </c>
+      <c r="B72" s="11" t="inlineStr">
+        <is>
+          <t>(this backfill)</t>
+        </is>
+      </c>
+      <c r="C72" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D72" s="11" t="inlineStr">
+        <is>
+          <t>(docs)</t>
+        </is>
+      </c>
+      <c r="E72" s="11" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="F72" s="11" t="inlineStr">
+        <is>
+          <t>Four-pillar audit (truth, cascade, hardcoded, duplicates) — all PASS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="11" t="inlineStr">
+        <is>
+          <t>S26b/pmt-reject-terminal</t>
+        </is>
+      </c>
+      <c r="B73" s="11" t="inlineStr">
+        <is>
+          <t>(this backfill)</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D73" s="11" t="inlineStr">
+        <is>
+          <t>(PMT lifecycle)</t>
+        </is>
+      </c>
+      <c r="E73" s="11" t="inlineStr">
+        <is>
+          <t>PMT, admin_console</t>
+        </is>
+      </c>
+      <c r="F73" s="11" t="inlineStr">
+        <is>
+          <t>Rejection now terminal; signoffs + audit row preserved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="11" t="inlineStr">
+        <is>
+          <t>S26b/pmt-config-live</t>
+        </is>
+      </c>
+      <c r="B74" s="11" t="inlineStr">
+        <is>
+          <t>(this backfill)</t>
+        </is>
+      </c>
+      <c r="C74" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D74" s="11" t="inlineStr">
+        <is>
+          <t>(PMT UI)</t>
+        </is>
+      </c>
+      <c r="E74" s="11" t="inlineStr">
+        <is>
+          <t>PMT, design</t>
+        </is>
+      </c>
+      <c r="F74" s="11" t="inlineStr">
+        <is>
+          <t>Configuration screen wired to /api/v1/admin/pmt/versions/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="11" t="inlineStr">
+        <is>
+          <t>S26b/approvals-queue</t>
+        </is>
+      </c>
+      <c r="B75" s="11" t="inlineStr">
+        <is>
+          <t>(this backfill)</t>
+        </is>
+      </c>
+      <c r="C75" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D75" s="11" t="inlineStr">
+        <is>
+          <t>(cross-module queue)</t>
+        </is>
+      </c>
+      <c r="E75" s="11" t="inlineStr">
+        <is>
+          <t>admin_console</t>
+        </is>
+      </c>
+      <c r="F75" s="11" t="inlineStr">
+        <is>
+          <t>Unified /api/v1/admin/approvals/ across CL, DQA, PMT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="11" t="inlineStr">
+        <is>
+          <t>S26b/admin-polish</t>
+        </is>
+      </c>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>(this backfill)</t>
+        </is>
+      </c>
+      <c r="C76" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D76" s="11" t="inlineStr">
+        <is>
+          <t>(admin UI)</t>
+        </is>
+      </c>
+      <c r="E76" s="11" t="inlineStr">
+        <is>
+          <t>admin_console, design</t>
+        </is>
+      </c>
+      <c r="F76" s="11" t="inlineStr">
+        <is>
+          <t>Null-safe DDUP, live CL detail, DQA descriptions, refdata-geography search reset.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: consent module manual page + sprint plan status (Epic 19 done)
- User manual: new modules/consent.md (purposes, states, endpoints, operator
  flows, the 7 downstream gates, DQA rules, go-live gates) + mkdocs nav entry.
- Sprint plan (08_sprint_plan.xlsx): S27+S28 Forward → Done; new Status session
  row for the consent build; Backlog Status rows for US-CONSENT-01..18 = Done;
  Story Map entries per wave; DEP-22/23/24 resolved (CONSENT-O-01/03/08 decided
  2026-05-30), DEP-25 partially resolved (citizen-portal stub delivered).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/08_sprint_plan.xlsx
+++ b/docs/08_sprint_plan.xlsx
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1523,6 +1523,36 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>S27→S28</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2026-05-30 → 2026-05-31</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>~1 day</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>23</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Consent Management module (Epic 19, US-CONSENT-01..18) — apps/consent behind CONSENT_MODULE_ENABLED. Catalogue + dual-approval, statement versioning, capture (walk-in/CAPI/Kobo + citizen portal), withdrawal flow + DPO queue + SLA sweep, gates into PMT/REF/DRS/DDUP/UPD/DIH/INT, audit chain, DQA rule pack, ADR-0024 + DPIA §14 + OpenAPI. Live-wired citizen screen (capture/withdraw/history) + per-purpose capture form + household Consent tab card. Also fixed pre-existing CI (bandit, JS, E004 check, dob matview migration, replica routing). 1820 py tests / 228 JS / 6-of-7 CI green; remaining pytest reds are pre-existing data_explorer/dqa debt (zero consent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1534,7 +1564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3977,6 +4007,230 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>S27/consent-foundation</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>28b7167</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>US-CONSENT-01/02/10/18</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>App scaffold, 8-table model, dual-approval catalogue, audit wiring, ADR-0024 + DPIA §14.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>S27/consent-rules-sla</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>b646e5b</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>US-CONSENT-07/09</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Consent (SEC), DAT-DQA</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>AC-CONSENT-* rule pack (DRAFT), SLA beat sweep, CONSENT-O-01 vocab reconcile (ELIGIBILITY).</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>S28/consent-propagation</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>c862b33</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>US-CONSENT-12/13/15/16</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>PMT, REF, DDUP, UPD</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Consent gates wired into PMT/REF/DDUP/UPD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>S28/consent-dih-dash</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>81b7da4</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>US-CONSENT-11/17</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>DIH, Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>DIH fast-track synthetic consent + DPO coverage stub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>S28/consent-drs</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>99c1541</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>US-CONSENT-14</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>API-DRS</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>DRS extract row-level consent gate (SQL).</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>S28/consent-frontend</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>4d4e13d..eef6e6b</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>US-CONSENT-03/05/08</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Consent (SEC), design</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Admin console screens + citizen portal + badge cluster + live-wired citizen screen + per-purpose capture form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>S28/consent-intake</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>278c54c, 581833f</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>US-CONSENT-03</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>INT, DIH</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Intake gate + capture (walk-in/CAPI/Kobo); capture form replaces legacy toggle.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3989,7 +4243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G120"/>
+  <dimension ref="A1:G138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -7952,6 +8206,672 @@
         </is>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>US-CONSENT-01</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Purpose catalogue CRUD + dual-approval; audit events; /api/v1/consent/purposes/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>US-CONSENT-02</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Statement versioning, i18n, one-ACTIVE-per-purpose partial index, is_material re-consent recount.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>US-CONSENT-03</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Intake capture: walk-in form per-purpose section + gate (refused→declined_consent); capture at promotion (web/CAPI/Kobo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>US-CONSENT-04</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Server-side capture + idempotency. Android/SQLCipher offline client is external (separate repo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>US-CONSENT-05</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Citizen dashboard live-wired to /api/v1/consent/members/{id}; matrix + withdraw.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>US-CONSENT-06</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Withdrawal flow, idempotent per day, 30-day SLA clock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>US-CONSENT-07</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>DPO withdrawal queue + decisions + bulk rules + hourly Celery SLA-breach sweep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>US-CONSENT-08</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Reusable ConsentBadgeCluster + per-purpose detail card on household Consent tab (with legacy inference).</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>US-CONSENT-09</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>AC-CONSENT-* DQA rule pack seeded DRAFT (scripts/seed_dqa_consent_rules.py); DPO ratifies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>US-CONSENT-10</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>AuditEvent per change + ConsentRecordVersion(audit_event_id); integrity = referential completeness (not a 2nd chain).</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>US-CONSENT-11</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>DIH fast-track synthetic consent from ratified DPA scope; unratified DPA holds promotion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>US-CONSENT-12</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>PMT recompute ELIGIBILITY gate; withdrawn/pending blocks + events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>US-CONSENT-13</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>REF send_referral gate on REFERRAL (blocks withdrawn/refused); blocked_member_ids helper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>US-CONSENT-14</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>DRS extract row-gate: render_bundle excludes blocked members per DSA consent_purposes (SQL layer).</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>US-CONSENT-15</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>DDUP merge reconciliation (union of grants; withdrawal wins; conflict blocks).</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>US-CONSENT-16</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>UPD head-change opens REGISTRATION re-capture sub-task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>US-CONSENT-17</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>DPO coverage dashboard stub — live KPI cards, charts deferred.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>US-CONSENT-18</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>PR #1 (Epic 19)</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>ADR-0024 + DPIA §14 + docs/openapi/consent.yaml.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G115"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7964,7 +8884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8271,6 +9191,60 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>S27</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Consent Management foundations: data model, purpose catalogue, statement versioning, intake capture (Web+CAPI), citizen dashboard, badge cluster, DQA rules, audit chain, DPIA addendum — delivered 2026-05-31 (PR #1, ADR-0024)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Consent (SEC), DAT-DQA, INT, SEC</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>US-CONSENT-01..05, US-CONSENT-08..10, US-CONSENT-18 (partial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>S28</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Consent propagation + withdrawal: ticket flow, DPO queue, DIH fast-track, PMT/REF/DRS/DDUP/UPD integration, coverage dashboard, ADR-0024 — delivered 2026-05-31 (PR #1, ADR-0024)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Consent (SEC), DIH, PMT, REF, API-DRS, DAT-DDUP, UPD, RPT</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>US-CONSENT-06, US-CONSENT-07, US-CONSENT-11..17, US-CONSENT-18 (close)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8282,7 +9256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8962,6 +9936,166 @@
       <c r="F21" t="inlineStr">
         <is>
           <t>Constrains the CAPI build-vs-buy choice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DEP-22</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>DPO sign-off on purpose catalogue (CONSENT-O-01)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>S27</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>DPO + MGLSD Legal</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>RESOLVED 2026-05-30: scope-doc 9 incl. ELIGIBILITY seeded (migration 0002). DPO production sign-off still required before flag-on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DEP-23</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>DPO sign-off on withdrawal SLA (CONSENT-O-03)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>S28</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>DPO + NSR Coordinator</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>RESOLVED 2026-05-30: 30 days adopted (DPPA §29). DPO production sign-off still required before flag-on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>DEP-24</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>DPA ratification model decision (CONSENT-O-08)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>S28</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>DPO + DIH team</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>RESOLVED 2026-05-30: one ratification at DPA activation. DIH fast-track (US-CONSENT-11) built to it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>DEP-25</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Citizen portal Keycloak realm</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>S27 (stub) / Release 3 (live)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>NSR MIS Architecture</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Partially resolved</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Stub auth delivered (citizen portal /portal/consent/). Keycloak realm still a Release-3 follow-up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>DEP-26</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Real translated statement copy (6 languages)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>S27</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>NSR Coordinator + DPO</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Statement v3 seeded with English real text + 6 placeholders flagged is_placeholder=True.</t>
         </is>
       </c>
     </row>
@@ -8986,7 +10120,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>NSR MIS Sprint Plan v0.2</t>
+          <t>NSR MIS Sprint Plan v0.3</t>
         </is>
       </c>
       <c r="B1" s="10" t="inlineStr"/>
@@ -8999,7 +10133,7 @@
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>15 May 2026</t>
+          <t>30 May 2026</t>
         </is>
       </c>
     </row>
@@ -9011,7 +10145,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>NSR MIS Architecture Team</t>
+          <t>Sprint Plan v0.2 (15 May 2026)</t>
         </is>
       </c>
     </row>

</xml_diff>